<commit_message>
feat(credit): expose credit cases list navigation to regular users across sidebar, credit search, and new registration
</commit_message>
<xml_diff>
--- a/public/downloads/credit_data_sources_catalog.xlsx
+++ b/public/downloads/credit_data_sources_catalog.xlsx
@@ -1,24 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8C087B7-41AE-44A7-9322-23C7BB99BEDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="データソース一覧" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="国交省ネガティブ情報仕様" state="visible" r:id="rId5"/>
+    <sheet name="データソース一覧" sheetId="1" r:id="rId1"/>
+    <sheet name="国交省ネガティブ情報仕様" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="100">
-  <si>
-    <t>Mieris 企業信用照会システム - 連携データソース＆取得情報カタログ</t>
-  </si>
-  <si>
-    <t>※本システムが取得・統合している公的確定データベースおよび民間ネットワークの全情報項目一覧</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="92">
   <si>
     <t>No</t>
   </si>
@@ -41,14 +39,14 @@
     <t>利用価値・調査用途</t>
   </si>
   <si>
-    <t xml:space="preserve">経済産業省
+    <t>経済産業省
 gBizINFO REST API</t>
   </si>
   <si>
     <t>公的法人プロファイル・届出公表情報</t>
   </si>
   <si>
-    <t xml:space="preserve">・法人名称（商号）・フリガナ
+    <t>・法人名称（商号）・フリガナ
 ・法人番号（13桁）
 ・代表者役職名 および 氏名
 ・本店所在地（住所）
@@ -57,18 +55,18 @@
 ・財務情報・表彰届出記録・特許出願情報</t>
   </si>
   <si>
-    <t xml:space="preserve">経済産業省 オープンデータ推進基盤
+    <t>経済産業省 オープンデータ推進基盤
 （公式REST API連携）</t>
   </si>
   <si>
-    <t xml:space="preserve">リアルタイム照会
+    <t>リアルタイム照会
 （社名入力サジェスト即時連動）</t>
   </si>
   <si>
     <t>取引先実態確認、同名企業誤認防止、代表者・事業規模の適正把握</t>
   </si>
   <si>
-    <t xml:space="preserve">国税庁
+    <t>国税庁
 法人番号公表サイト ＆
 適格請求書（インボイス）公表システム</t>
   </si>
@@ -76,7 +74,7 @@
     <t>公的法人登記・閉鎖・税務適格性</t>
   </si>
   <si>
-    <t xml:space="preserve">・法人番号（13桁）の適法性・存在確認
+    <t>・法人番号（13桁）の適法性・存在確認
 ・登記記録の閉鎖状況（存続 / 閉鎖・清算結了・解散）
 ・登記記録閉鎖年月日 および 閉鎖事由
 ・インボイス登録番号（T+13桁）の有効性
@@ -84,50 +82,50 @@
 ・モジュラス9/11公式検査数字（チェックディジット）適合判定</t>
   </si>
   <si>
-    <t xml:space="preserve">国税庁 法人番号法・消費税法
+    <t>国税庁 法人番号法・消費税法
 （API / チェックディジットエンジン）</t>
   </si>
   <si>
-    <t xml:space="preserve">リアルタイム照会
+    <t>リアルタイム照会
 （検索時即時バリデーション）</t>
   </si>
   <si>
     <t>偽装インボイス防止、倒産・登記閉鎖企業の検知、架空企業排除</t>
   </si>
   <si>
-    <t xml:space="preserve">厚生労働省
+    <t>厚生労働省
 労働基準関係法令違反 送検公表データ</t>
   </si>
   <si>
     <t>労働基準法違反・ブラック企業公表事案</t>
   </si>
   <si>
-    <t xml:space="preserve">・送検公表日 / 管轄労働局・労働基準監督署名
+    <t>・送検公表日 / 管轄労働局・労働基準監督署名
 ・被疑者氏名・違反法条（労基法第24条賃金不払、最賃法違反、安衛法等）
 ・違反行為・不払いの具体的事案概要
 ・未払い被害金額（公表された不払賃金・割増手当概算額）
 ・公表事案ステータス（送検確定事実）</t>
   </si>
   <si>
-    <t xml:space="preserve">厚生労働省 労働基準法・最低賃金法
+    <t>厚生労働省 労働基準法・最低賃金法
 （公表リスト定期自動同期）</t>
   </si>
   <si>
-    <t xml:space="preserve">毎週月曜 4:00 (JST) 自動同期
+    <t>毎週月曜 4:00 (JST) 自動同期
 ＋ 管理画面ワンクリック同期</t>
   </si>
   <si>
     <t>下請代金・人件費踏み倒し常習企業の排除、労務コンプライアンス判定</t>
   </si>
   <si>
-    <t xml:space="preserve">国土交通省・管轄各自治体
+    <t>国土交通省・管轄各自治体
 ネガティブ情報等検索システム</t>
   </si>
   <si>
     <t>建設業・宅建・建築基準監督処分記録</t>
   </si>
   <si>
-    <t xml:space="preserve">・処分等発令年月日 / 担当行政機関（国交省各地方整備局、各都道府県知事等）
+    <t>・処分等発令年月日 / 担当行政機関（国交省各地方整備局、各都道府県知事等）
 ・事業者名・法人番号・免許/許可登録番号
 ・本社住所
 ・処分の種類（業務停止、免許取消、是正指示、許可取消等）
@@ -136,25 +134,25 @@
 ・違反行為の具体概要（融資資料偽装、重要事項不実説明、界壁施工不備等）</t>
   </si>
   <si>
-    <t xml:space="preserve">国土交通省 各業法ネガティブ情報公表指針
+    <t>国土交通省 各業法ネガティブ情報公表指針
 （検索CGIデータ連携）</t>
   </si>
   <si>
-    <t xml:space="preserve">定期バッチ同期
+    <t>定期バッチ同期
 （公表期間: 原則5年間保管）</t>
   </si>
   <si>
     <t>不動産取引・建築・元請け取引の安全性検証、不正・改ざん企業排除</t>
   </si>
   <si>
-    <t xml:space="preserve">消費者庁
+    <t>消費者庁
 特定商取引法・景品表示法 行政処分</t>
   </si>
   <si>
     <t>特商法・景表法 確定行政処分記録</t>
   </si>
   <si>
-    <t xml:space="preserve">・措置・命令発令日 / 管轄課（取引対策課・表示対策課）
+    <t>・措置・命令発令日 / 管轄課（取引対策課・表示対策課）
 ・事業者名・所在地・代表者名
 ・適用法令（特商法第8条第1項、景表法第7条等）
 ・処分区分（業務停止命令、指示処分、課徴金納付命令、再発防止措置等）
@@ -162,7 +160,7 @@
 ・違反事実の具体的内容（不実告知、誇大広告、定期購入詐欺的表示等）</t>
   </si>
   <si>
-    <t xml:space="preserve">消費者庁 特定商取引法・景品表示法
+    <t>消費者庁 特定商取引法・景品表示法
 （公表資料連携）</t>
   </si>
   <si>
@@ -172,14 +170,14 @@
     <t>悪質マーケティング・詐欺的取引企業の検知、企業倫理リスク判定</t>
   </si>
   <si>
-    <t xml:space="preserve">国立印刷局「官報」公告 ＆
+    <t>国立印刷局「官報」公告 ＆
 管轄地方裁判所</t>
   </si>
   <si>
     <t>裁判所公認 破産・倒産公告記録</t>
   </si>
   <si>
-    <t xml:space="preserve">・官報掲載日 / 担当裁判所（東京地方裁判所民事第20部等）
+    <t>・官報掲載日 / 担当裁判所（東京地方裁判所民事第20部等）
 ・事件番号（令和◯年(フ)第◯号 等）
 ・法的手続種別（破産手続開始、民事再生、特別清算、会社更生等）
 ・主文（破産手続開始決定、廃止決定等）
@@ -187,7 +185,7 @@
 ・債権届出期間・財産状況報告集会期日</t>
   </si>
   <si>
-    <t xml:space="preserve">最高裁判所・破産法・民事再生法
+    <t>最高裁判所・破産法・民事再生法
 国立印刷局 インターネット版官報</t>
   </si>
   <si>
@@ -197,39 +195,9 @@
     <t>法的倒産・債務整理企業の確実な把握、回収不能リスクの事前回避</t>
   </si>
   <si>
-    <t xml:space="preserve">本システム独自ネットワーク
-加盟企業間 信用情報共有NW</t>
-  </si>
-  <si>
-    <t>民間取引先 債権未払い・支払遅延被害申告</t>
-  </si>
-  <si>
-    <t xml:space="preserve">・未払い請求金額（税込）
-・当初支払期日 および 支払遅延日数
-・入金ステータス（未払い継続中 / 和解・遅延解決・回収完了）
-・客観的証憑（発注書、納品書、請求書、支払期日通知書、督促履歴）
-・取引の経緯 および 相手方の主張
-・相手先営業実態（連絡可能協議中 / 音信不通 / 事務所退去 / 弁護士受任等）
-・情報登録企業名（加盟企業）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">加盟企業間 信用情報共有規約
-（事前同意書取得・客観証憑審査制）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">加盟企業による都度登録
-（運営管理者による証憑審査承認後公開）</t>
-  </si>
-  <si>
-    <t>公的処分に至る前の初期支払遅延・未回収リスク検知、連鎖倒産防止</t>
-  </si>
-  <si>
     <t>国土交通省 ネガティブ情報等検索サイト（https://www.mlit.go.jp/nega-inf/）連携仕様</t>
   </si>
   <si>
-    <t>※調査結果: POST/GETリクエストによるHTMLスクレイピングにて全項目完全自動取得可能（CAPTCHAなし・UTF-8）</t>
-  </si>
-  <si>
     <t>業種・分野名</t>
   </si>
   <si>
@@ -369,75 +337,96 @@
   </si>
   <si>
     <t>処分年月日、運輸局名、事業者名、営業所名、車両使用停止(日車数)、違反点数、過労運転・未点呼等概要</t>
+  </si>
+  <si>
+    <t>Mieris連携データソース＆取得情報カタログ</t>
+    <phoneticPr fontId="10"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="11" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="11">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="14"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="14"/>
       <name val="Meiryo UI"/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="FF475569"/>
-      <sz val="9"/>
-      <name val="Meiryo UI"/>
+      <family val="3"/>
+      <charset val="128"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
       <name val="Meiryo UI"/>
+      <family val="3"/>
+      <charset val="128"/>
     </font>
     <font>
       <sz val="9"/>
       <name val="Meiryo UI"/>
+      <family val="3"/>
+      <charset val="128"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Meiryo UI"/>
+      <family val="3"/>
+      <charset val="128"/>
     </font>
     <font>
       <b/>
+      <sz val="9"/>
       <color rgb="FF1E293B"/>
-      <sz val="9"/>
       <name val="Meiryo UI"/>
+      <family val="3"/>
+      <charset val="128"/>
     </font>
     <font>
       <b/>
+      <sz val="13"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="13"/>
       <name val="Meiryo UI"/>
+      <family val="3"/>
+      <charset val="128"/>
     </font>
     <font>
       <b/>
+      <sz val="9"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="9"/>
       <name val="Meiryo UI"/>
+      <family val="3"/>
+      <charset val="128"/>
     </font>
     <font>
       <b/>
+      <sz val="9"/>
       <color rgb="FF0284C7"/>
-      <sz val="9"/>
       <name val="Consolas"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <name val="Meiryo UI"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="6"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="7">
@@ -454,11 +443,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF1F5F9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF0F172A"/>
       </patternFill>
     </fill>
@@ -470,6 +454,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF0284C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -515,80 +505,83 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="標準" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -924,9 +917,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
@@ -937,226 +930,192 @@
     <col min="7" max="7" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" ht="32.1" customHeight="1">
+      <c r="A1" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+    </row>
+    <row r="2" spans="1:7" s="1" customFormat="1" ht="27.95" customHeight="1">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-    </row>
-    <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-    </row>
-    <row r="3" ht="28" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="E2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="F2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="G2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="4" t="s">
+    </row>
+    <row r="3" spans="1:7" s="3" customFormat="1" ht="110.1" customHeight="1">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="C3" s="6" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" ht="110" customHeight="1" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="6">
-        <v>1</v>
-      </c>
-      <c r="B4" s="7" t="s">
+      <c r="D3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="E3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="F3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="G3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="8" t="s">
+    </row>
+    <row r="4" spans="1:7" s="3" customFormat="1" ht="110.1" customHeight="1">
+      <c r="A4" s="7">
+        <v>2</v>
+      </c>
+      <c r="B4" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="C4" s="9" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="5" ht="110" customHeight="1" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="9">
-        <v>2</v>
-      </c>
-      <c r="B5" s="10" t="s">
+      <c r="D4" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="E4" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="F4" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="G4" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="11" t="s">
+    </row>
+    <row r="5" spans="1:7" s="3" customFormat="1" ht="110.1" customHeight="1">
+      <c r="A5" s="4">
+        <v>3</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="C5" s="6" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" ht="110" customHeight="1" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="6">
-        <v>3</v>
-      </c>
-      <c r="B6" s="7" t="s">
+      <c r="D5" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="E5" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="F5" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="G5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="8" t="s">
+    </row>
+    <row r="6" spans="1:7" s="3" customFormat="1" ht="110.1" customHeight="1">
+      <c r="A6" s="7">
+        <v>4</v>
+      </c>
+      <c r="B6" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="C6" s="24" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="7" ht="110" customHeight="1" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="9">
-        <v>4</v>
-      </c>
-      <c r="B7" s="10" t="s">
+      <c r="D6" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="E6" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="F6" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="G6" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="F7" s="11" t="s">
+    </row>
+    <row r="7" spans="1:7" s="3" customFormat="1" ht="110.1" customHeight="1">
+      <c r="A7" s="4">
+        <v>5</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="C7" s="6" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="8" ht="110" customHeight="1" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="6">
-        <v>5</v>
-      </c>
-      <c r="B8" s="7" t="s">
+      <c r="D7" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="E7" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="F7" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="G7" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="F8" s="8" t="s">
+    </row>
+    <row r="8" spans="1:7" s="3" customFormat="1" ht="110.1" customHeight="1">
+      <c r="A8" s="7">
+        <v>6</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="C8" s="9" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="9" ht="110" customHeight="1" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="9">
-        <v>6</v>
-      </c>
-      <c r="B9" s="10" t="s">
+      <c r="D8" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="E8" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="F8" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="G8" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="F9" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="G9" s="11" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="10" ht="110" customHeight="1" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="6">
-        <v>7</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>50</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
   </mergeCells>
+  <phoneticPr fontId="10"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F12"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -1166,232 +1125,222 @@
     <col min="6" max="6" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:6" ht="30" customHeight="1">
+      <c r="A1" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+    </row>
+    <row r="2" spans="1:6" s="10" customFormat="1" ht="26.1" customHeight="1">
+      <c r="A2" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" s="12" customFormat="1" ht="42" customHeight="1">
+      <c r="A3" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-    </row>
-    <row r="2" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="C3" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-    </row>
-    <row r="3" ht="26" customHeight="1" spans="1:6" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="D3" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="E3" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="F3" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="D3" s="14" t="s">
+    </row>
+    <row r="4" spans="1:6" s="12" customFormat="1" ht="42" customHeight="1">
+      <c r="A4" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="B4" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="C4" s="17" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="4" ht="42" customHeight="1" spans="1:6" s="15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
+      <c r="D4" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="E4" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="F4" s="20" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="12" customFormat="1" ht="42" customHeight="1">
+      <c r="A5" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="B5" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="C5" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="D5" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="E5" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F5" s="16" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="12" customFormat="1" ht="42" customHeight="1">
+      <c r="A6" s="17" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="5" ht="42" customHeight="1" spans="1:6" s="15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="20" t="s">
+      <c r="B6" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="B5" s="21" t="s">
+      <c r="C6" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="D6" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="E6" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="D5" s="22" t="s">
-        <v>62</v>
-      </c>
-      <c r="E5" s="20" t="s">
+      <c r="F6" s="20" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="12" customFormat="1" ht="42" customHeight="1">
+      <c r="A7" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="F5" s="23" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="6" ht="42" customHeight="1" spans="1:6" s="15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="16" t="s">
+      <c r="B7" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="C7" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="D7" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="E7" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="D6" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="E6" s="16" t="s">
+      <c r="F7" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F6" s="19" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="7" ht="42" customHeight="1" spans="1:6" s="15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="20" t="s">
+    </row>
+    <row r="8" spans="1:6" s="12" customFormat="1" ht="42" customHeight="1">
+      <c r="A8" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="B7" s="21" t="s">
+      <c r="B8" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="C7" s="20" t="s">
+      <c r="C8" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="D7" s="22" t="s">
-        <v>62</v>
-      </c>
-      <c r="E7" s="20" t="s">
+      <c r="D8" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="E8" s="17" t="s">
         <v>76</v>
       </c>
-      <c r="F7" s="23" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="8" ht="42" customHeight="1" spans="1:6" s="15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="16" t="s">
+      <c r="F8" s="20" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="12" customFormat="1" ht="42" customHeight="1">
+      <c r="A9" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B9" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C9" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="D8" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="E8" s="16" t="s">
+      <c r="D9" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="E9" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="F9" s="16" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="12" customFormat="1" ht="42" customHeight="1">
+      <c r="A10" s="17" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="9" ht="42" customHeight="1" spans="1:6" s="15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="20" t="s">
+      <c r="B10" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="C10" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="C9" s="20" t="s">
+      <c r="D10" s="19" t="s">
         <v>84</v>
       </c>
-      <c r="D9" s="22" t="s">
-        <v>62</v>
-      </c>
-      <c r="E9" s="20" t="s">
+      <c r="E10" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="F9" s="23" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="10" ht="42" customHeight="1" spans="1:6" s="15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="16" t="s">
+      <c r="F10" s="20" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" s="12" customFormat="1" ht="42" customHeight="1">
+      <c r="A11" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B11" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C11" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="D10" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="E10" s="16" t="s">
+      <c r="D11" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="F10" s="19" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="11" ht="42" customHeight="1" spans="1:6" s="15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="20" t="s">
+      <c r="E11" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="B11" s="21" t="s">
-        <v>91</v>
-      </c>
-      <c r="C11" s="20" t="s">
-        <v>92</v>
-      </c>
-      <c r="D11" s="22" t="s">
-        <v>93</v>
-      </c>
-      <c r="E11" s="20" t="s">
-        <v>94</v>
-      </c>
-      <c r="F11" s="23" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="12" ht="42" customHeight="1" spans="1:6" s="15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="16" t="s">
-        <v>95</v>
-      </c>
-      <c r="B12" s="17" t="s">
-        <v>96</v>
-      </c>
-      <c r="C12" s="16" t="s">
-        <v>97</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="E12" s="16" t="s">
-        <v>99</v>
-      </c>
-      <c r="F12" s="19" t="s">
-        <v>81</v>
+      <c r="F11" s="16" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
   </mergeCells>
+  <phoneticPr fontId="10"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>